<commit_message>
Refresh Google Scholar statistics
</commit_message>
<xml_diff>
--- a/assets/data/scholar-citations.xlsx
+++ b/assets/data/scholar-citations.xlsx
@@ -7,8 +7,8 @@
     <sheet name="逐篇论文" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'每日引用'!$A$1:$F$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'逐篇论文'!$A$1:$F$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'每日引用'!$A$1:$F$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'逐篇论文'!$A$1:$F$112</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -385,7 +385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -623,11 +623,31 @@
         <v>28</v>
       </c>
       <c r="F11" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="15" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>8978</v>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>46296.66398726479</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F11"/>
+  <autoFilter ref="A1:F12"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -638,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1516,7 +1536,7 @@
         <v>0</v>
       </c>
       <c r="F39" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="40" ht="42" customHeight="1">
@@ -1540,7 +1560,7 @@
         <v>0</v>
       </c>
       <c r="F40" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="41" ht="42" customHeight="1">
@@ -1564,7 +1584,7 @@
         <v>2</v>
       </c>
       <c r="F41" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="42" ht="42" customHeight="1">
@@ -1588,7 +1608,7 @@
         <v>2</v>
       </c>
       <c r="F42" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="43" ht="42" customHeight="1">
@@ -1612,7 +1632,7 @@
         <v>5</v>
       </c>
       <c r="F43" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="44" ht="42" customHeight="1">
@@ -1636,7 +1656,7 @@
         <v>0</v>
       </c>
       <c r="F44" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="45" ht="42" customHeight="1">
@@ -1660,7 +1680,7 @@
         <v>2</v>
       </c>
       <c r="F45" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="46" ht="42" customHeight="1">
@@ -1684,7 +1704,7 @@
         <v>0</v>
       </c>
       <c r="F46" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="47" ht="42" customHeight="1">
@@ -1708,7 +1728,7 @@
         <v>1</v>
       </c>
       <c r="F47" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="48" ht="42" customHeight="1">
@@ -1732,7 +1752,7 @@
         <v>8</v>
       </c>
       <c r="F48" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="49" ht="42" customHeight="1">
@@ -1756,7 +1776,7 @@
         <v>1</v>
       </c>
       <c r="F49" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="50" ht="42" customHeight="1">
@@ -1780,7 +1800,7 @@
         <v>2</v>
       </c>
       <c r="F50" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="51" ht="42" customHeight="1">
@@ -1804,7 +1824,7 @@
         <v>9</v>
       </c>
       <c r="F51" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="52" ht="42" customHeight="1">
@@ -1828,7 +1848,7 @@
         <v>1</v>
       </c>
       <c r="F52" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="53" ht="42" customHeight="1">
@@ -1852,7 +1872,7 @@
         <v>8</v>
       </c>
       <c r="F53" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="54" ht="42" customHeight="1">
@@ -1876,7 +1896,7 @@
         <v>0</v>
       </c>
       <c r="F54" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="55" ht="42" customHeight="1">
@@ -1900,7 +1920,7 @@
         <v>3</v>
       </c>
       <c r="F55" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="56" ht="42" customHeight="1">
@@ -1924,7 +1944,7 @@
         <v>1</v>
       </c>
       <c r="F56" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="57" ht="42" customHeight="1">
@@ -1948,7 +1968,7 @@
         <v>1</v>
       </c>
       <c r="F57" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="58" ht="42" customHeight="1">
@@ -1972,7 +1992,7 @@
         <v>1</v>
       </c>
       <c r="F58" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="59" ht="42" customHeight="1">
@@ -1996,7 +2016,7 @@
         <v>0</v>
       </c>
       <c r="F59" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="60" ht="42" customHeight="1">
@@ -2020,7 +2040,7 @@
         <v>0</v>
       </c>
       <c r="F60" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="61" ht="42" customHeight="1">
@@ -2044,7 +2064,7 @@
         <v>18</v>
       </c>
       <c r="F61" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="62" ht="42" customHeight="1">
@@ -2068,7 +2088,7 @@
         <v>1</v>
       </c>
       <c r="F62" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="63" ht="42" customHeight="1">
@@ -2092,7 +2112,7 @@
         <v>8</v>
       </c>
       <c r="F63" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="64" ht="42" customHeight="1">
@@ -2116,7 +2136,7 @@
         <v>21</v>
       </c>
       <c r="F64" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="65" ht="42" customHeight="1">
@@ -2140,7 +2160,7 @@
         <v>0</v>
       </c>
       <c r="F65" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="66" ht="42" customHeight="1">
@@ -2164,7 +2184,7 @@
         <v>1</v>
       </c>
       <c r="F66" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="67" ht="42" customHeight="1">
@@ -2188,7 +2208,7 @@
         <v>5</v>
       </c>
       <c r="F67" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="68" ht="42" customHeight="1">
@@ -2212,7 +2232,7 @@
         <v>4</v>
       </c>
       <c r="F68" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="69" ht="42" customHeight="1">
@@ -2236,7 +2256,7 @@
         <v>6</v>
       </c>
       <c r="F69" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="70" ht="42" customHeight="1">
@@ -2260,7 +2280,7 @@
         <v>0</v>
       </c>
       <c r="F70" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="71" ht="42" customHeight="1">
@@ -2284,7 +2304,7 @@
         <v>25</v>
       </c>
       <c r="F71" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="72" ht="42" customHeight="1">
@@ -2308,7 +2328,7 @@
         <v>1</v>
       </c>
       <c r="F72" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="73" ht="42" customHeight="1">
@@ -2332,7 +2352,7 @@
         <v>11</v>
       </c>
       <c r="F73" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="74" ht="42" customHeight="1">
@@ -2356,7 +2376,7 @@
         <v>1</v>
       </c>
       <c r="F74" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
       </c>
     </row>
     <row r="75" ht="42" customHeight="1">
@@ -2380,11 +2400,899 @@
         <v>1</v>
       </c>
       <c r="F75" s="17" t="n">
-        <v>46293.66112145912</v>
+        <v>46293.66112145833</v>
+      </c>
+    </row>
+    <row r="76" ht="42" customHeight="1">
+      <c r="A76" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B76" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:-_dYPAW6P2MC</t>
+        </is>
+      </c>
+      <c r="C76" s="20" t="inlineStr">
+        <is>
+          <t>AnyMatch: Supercharging Universal Multi-modal Image Matching with Large-Scale Single-View Images</t>
+        </is>
+      </c>
+      <c r="D76" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="77" ht="42" customHeight="1">
+      <c r="A77" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B77" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:_Ybze24A_UAC</t>
+        </is>
+      </c>
+      <c r="C77" s="20" t="inlineStr">
+        <is>
+          <t>ArgMatch: Adaptive Refinement Gathering for Efficient Dense Matching</t>
+        </is>
+      </c>
+      <c r="D77" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E77" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="78" ht="42" customHeight="1">
+      <c r="A78" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B78" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:1yQoGdGgb4wC</t>
+        </is>
+      </c>
+      <c r="C78" s="20" t="inlineStr">
+        <is>
+          <t>C2RF: Bridging Multi-modal Image Registration and Fusion via Commonality Mining and Contrastive Learning</t>
+        </is>
+      </c>
+      <c r="D78" s="16" t="n">
+        <v>80</v>
+      </c>
+      <c r="E78" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="79" ht="42" customHeight="1">
+      <c r="A79" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B79" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:WA5NYHcadZ8C</t>
+        </is>
+      </c>
+      <c r="C79" s="20" t="inlineStr">
+        <is>
+          <t>CAMF: An interpretable infrared and visible image fusion network based on class activation mapping</t>
+        </is>
+      </c>
+      <c r="D79" s="16" t="n">
+        <v>107</v>
+      </c>
+      <c r="E79" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F79" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="80" ht="42" customHeight="1">
+      <c r="A80" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B80" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:W5xh706n7nkC</t>
+        </is>
+      </c>
+      <c r="C80" s="20" t="inlineStr">
+        <is>
+          <t>CLTE: Infrared and visible image fusion through cross-domain learning and texture-contrast enhancement</t>
+        </is>
+      </c>
+      <c r="D80" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="E80" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="81" ht="42" customHeight="1">
+      <c r="A81" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B81" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:ZuybSZzF8UAC</t>
+        </is>
+      </c>
+      <c r="C81" s="20" t="inlineStr">
+        <is>
+          <t>Comatch: Dynamic covisibility-aware transformer for bilateral subpixel-level semi-dense image matching</t>
+        </is>
+      </c>
+      <c r="D81" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="E81" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="82" ht="42" customHeight="1">
+      <c r="A82" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B82" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:Fu2w8maKXqMC</t>
+        </is>
+      </c>
+      <c r="C82" s="20" t="inlineStr">
+        <is>
+          <t>Controlfusion: A controllable image fusion network with language-vision degradation prompts</t>
+        </is>
+      </c>
+      <c r="D82" s="16" t="n">
+        <v>41</v>
+      </c>
+      <c r="E82" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="83" ht="42" customHeight="1">
+      <c r="A83" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B83" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:dQ2og3OwTAUC</t>
+        </is>
+      </c>
+      <c r="C83" s="20" t="inlineStr">
+        <is>
+          <t>Deep learning reforms image matching: A survey and outlook</t>
+        </is>
+      </c>
+      <c r="D83" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="E83" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="84" ht="42" customHeight="1">
+      <c r="A84" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B84" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:35r97b3x0nAC</t>
+        </is>
+      </c>
+      <c r="C84" s="20" t="inlineStr">
+        <is>
+          <t>Deep learning-based image fusion: A survey</t>
+        </is>
+      </c>
+      <c r="D84" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="E84" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="85" ht="42" customHeight="1">
+      <c r="A85" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B85" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:tkaPQYYpVKoC</t>
+        </is>
+      </c>
+      <c r="C85" s="20" t="inlineStr">
+        <is>
+          <t>Diff-IF: Multi-modality image fusion via diffusion model with fusion knowledge prior</t>
+        </is>
+      </c>
+      <c r="D85" s="16" t="n">
+        <v>267</v>
+      </c>
+      <c r="E85" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="86" ht="42" customHeight="1">
+      <c r="A86" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B86" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:tKAzc9rXhukC</t>
+        </is>
+      </c>
+      <c r="C86" s="20" t="inlineStr">
+        <is>
+          <t>Diff-MEF: Cross-Modal Diffusion Framework With Text Prompts and Semantic Perception for Multi-Exposure Image Fusion</t>
+        </is>
+      </c>
+      <c r="D86" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E86" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="87" ht="42" customHeight="1">
+      <c r="A87" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B87" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:PR6Y55bgFSsC</t>
+        </is>
+      </c>
+      <c r="C87" s="20" t="inlineStr">
+        <is>
+          <t>Diff-Retinex++: Retinex-driven reinforced diffusion model for low-light image enhancement</t>
+        </is>
+      </c>
+      <c r="D87" s="16" t="n">
+        <v>86</v>
+      </c>
+      <c r="E87" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="88" ht="42" customHeight="1">
+      <c r="A88" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B88" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:t6usbXjVLHcC</t>
+        </is>
+      </c>
+      <c r="C88" s="20" t="inlineStr">
+        <is>
+          <t>Diff-retinex: Rethinking low-light image enhancement with a generative diffusion model</t>
+        </is>
+      </c>
+      <c r="D88" s="16" t="n">
+        <v>473</v>
+      </c>
+      <c r="E88" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="89" ht="42" customHeight="1">
+      <c r="A89" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B89" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:JoZmwDi-zQgC</t>
+        </is>
+      </c>
+      <c r="C89" s="20" t="inlineStr">
+        <is>
+          <t>Dispel darkness for better fusion: A controllable visual enhancer based on cross-modal conditional adversarial learning</t>
+        </is>
+      </c>
+      <c r="D89" s="16" t="n">
+        <v>65</v>
+      </c>
+      <c r="E89" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="90" ht="42" customHeight="1">
+      <c r="A90" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B90" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:J-pR_7NvFogC</t>
+        </is>
+      </c>
+      <c r="C90" s="20" t="inlineStr">
+        <is>
+          <t>DIVFusion: Darkness-free infrared and visible image fusion</t>
+        </is>
+      </c>
+      <c r="D90" s="16" t="n">
+        <v>606</v>
+      </c>
+      <c r="E90" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="91" ht="42" customHeight="1">
+      <c r="A91" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B91" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:q3oQSFYPqjQC</t>
+        </is>
+      </c>
+      <c r="C91" s="20" t="inlineStr">
+        <is>
+          <t>DRLIE: Flexible low-light image enhancement via disentangled representations</t>
+        </is>
+      </c>
+      <c r="D91" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="E91" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="92" ht="42" customHeight="1">
+      <c r="A92" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B92" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:SdhP9T11ey4C</t>
+        </is>
+      </c>
+      <c r="C92" s="20" t="inlineStr">
+        <is>
+          <t>DRMF: Degradation-Robust Multi-Modal Image Fusion via Composable Diffusion Prior</t>
+        </is>
+      </c>
+      <c r="D92" s="16" t="n">
+        <v>104</v>
+      </c>
+      <c r="E92" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F92" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="93" ht="42" customHeight="1">
+      <c r="A93" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B93" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:ye4kPcJQO24C</t>
+        </is>
+      </c>
+      <c r="C93" s="20" t="inlineStr">
+        <is>
+          <t>DSPFusion: Image fusion via degradation and semantic dual-prior guidance</t>
+        </is>
+      </c>
+      <c r="D93" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="E93" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="94" ht="42" customHeight="1">
+      <c r="A94" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B94" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:j8SEvjWlNXcC</t>
+        </is>
+      </c>
+      <c r="C94" s="20" t="inlineStr">
+        <is>
+          <t>From single-modal to multi-modal: A survey and perspective on adversarial attacks in multi-modal visual systems</t>
+        </is>
+      </c>
+      <c r="D94" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F94" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="95" ht="42" customHeight="1">
+      <c r="A95" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B95" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:fEOibwPWpKIC</t>
+        </is>
+      </c>
+      <c r="C95" s="20" t="inlineStr">
+        <is>
+          <t>GText-IF: Leveraging Text-Driven Semantics for Degradation-Aware Image Fusion</t>
+        </is>
+      </c>
+      <c r="D95" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F95" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="96" ht="42" customHeight="1">
+      <c r="A96" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B96" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:7T2F9Uy0os0C</t>
+        </is>
+      </c>
+      <c r="C96" s="20" t="inlineStr">
+        <is>
+          <t>GTMFuse: Group-attention transformer-driven multiscale dense feature-enhanced network for infrared and visible image fusion</t>
+        </is>
+      </c>
+      <c r="D96" s="16" t="n">
+        <v>69</v>
+      </c>
+      <c r="E96" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="97" ht="42" customHeight="1">
+      <c r="A97" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B97" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:_Re3VWB3Y0AC</t>
+        </is>
+      </c>
+      <c r="C97" s="20" t="inlineStr">
+        <is>
+          <t>Human-machine collaboration in reshaping visual perception and cognition</t>
+        </is>
+      </c>
+      <c r="D97" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E97" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F97" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="98" ht="42" customHeight="1">
+      <c r="A98" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B98" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:5Ul4iDaHHb8C</t>
+        </is>
+      </c>
+      <c r="C98" s="20" t="inlineStr">
+        <is>
+          <t>Image fusion in the loop of high-level vision tasks: A semantic-aware real-time infrared and visible image fusion network</t>
+        </is>
+      </c>
+      <c r="D98" s="16" t="n">
+        <v>1296</v>
+      </c>
+      <c r="E98" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F98" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="99" ht="42" customHeight="1">
+      <c r="A99" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B99" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:BrmTIyaxlBUC</t>
+        </is>
+      </c>
+      <c r="C99" s="20" t="inlineStr">
+        <is>
+          <t>Infrared and visible image fusion via parallel scene and texture learning</t>
+        </is>
+      </c>
+      <c r="D99" s="16" t="n">
+        <v>73</v>
+      </c>
+      <c r="E99" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="100" ht="42" customHeight="1">
+      <c r="A100" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B100" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:uLbwQdceFCQC</t>
+        </is>
+      </c>
+      <c r="C100" s="20" t="inlineStr">
+        <is>
+          <t>Mask-DiFuser: A masked diffusion model for unified unsupervised image fusion</t>
+        </is>
+      </c>
+      <c r="D100" s="16" t="n">
+        <v>82</v>
+      </c>
+      <c r="E100" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F100" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="101" ht="42" customHeight="1">
+      <c r="A101" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B101" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:VOx2b1Wkg3QC</t>
+        </is>
+      </c>
+      <c r="C101" s="20" t="inlineStr">
+        <is>
+          <t>PIAFusion: A progressive infrared and visible image fusion network based on illumination aware</t>
+        </is>
+      </c>
+      <c r="D101" s="16" t="n">
+        <v>1427</v>
+      </c>
+      <c r="E101" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F101" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="102" ht="42" customHeight="1">
+      <c r="A102" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B102" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:Mojj43d5GZwC</t>
+        </is>
+      </c>
+      <c r="C102" s="20" t="inlineStr">
+        <is>
+          <t>PTET: A progressive token exchanging transformer for infrared and visible image fusion</t>
+        </is>
+      </c>
+      <c r="D102" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="E102" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F102" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="103" ht="42" customHeight="1">
+      <c r="A103" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B103" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:2KloaMYe4IUC</t>
+        </is>
+      </c>
+      <c r="C103" s="20" t="inlineStr">
+        <is>
+          <t>ReCoFuse: Ultra-Robust Image Fusion via Restorative Multi-Modal Diffusion Reciprocal Coupling</t>
+        </is>
+      </c>
+      <c r="D103" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E103" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F103" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="104" ht="42" customHeight="1">
+      <c r="A104" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B104" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:XiVPGOgt02cC</t>
+        </is>
+      </c>
+      <c r="C104" s="20" t="inlineStr">
+        <is>
+          <t>Rethinking the necessity of image fusion in high-level vision tasks: A practical infrared and visible image fusion network based on progressive semantic injection and scene …</t>
+        </is>
+      </c>
+      <c r="D104" s="16" t="n">
+        <v>464</v>
+      </c>
+      <c r="E104" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F104" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="105" ht="42" customHeight="1">
+      <c r="A105" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B105" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:geHnlv5EZngC</t>
+        </is>
+      </c>
+      <c r="C105" s="20" t="inlineStr">
+        <is>
+          <t>STDFusionNet: An infrared and visible image fusion network based on salient target detection</t>
+        </is>
+      </c>
+      <c r="D105" s="16" t="n">
+        <v>718</v>
+      </c>
+      <c r="E105" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F105" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="106" ht="42" customHeight="1">
+      <c r="A106" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B106" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:wbdj-CoPYUoC</t>
+        </is>
+      </c>
+      <c r="C106" s="20" t="inlineStr">
+        <is>
+          <t>SuperFusion: A versatile image registration and fusion network with semantic awareness</t>
+        </is>
+      </c>
+      <c r="D106" s="16" t="n">
+        <v>553</v>
+      </c>
+      <c r="E106" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F106" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="107" ht="42" customHeight="1">
+      <c r="A107" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B107" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:tzM49s52ZIMC</t>
+        </is>
+      </c>
+      <c r="C107" s="20" t="inlineStr">
+        <is>
+          <t>Supplementary Material of “VideoFusion: A Spatio-Temporal Collaborative Network for Multi-modal Video Fusion”</t>
+        </is>
+      </c>
+      <c r="D107" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="108" ht="42" customHeight="1">
+      <c r="A108" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B108" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:eJXPG6dFmWUC</t>
+        </is>
+      </c>
+      <c r="C108" s="20" t="inlineStr">
+        <is>
+          <t>SwinFusion: Cross-domain long-range learning for general image fusion via swin transformer</t>
+        </is>
+      </c>
+      <c r="D108" s="16" t="n">
+        <v>1775</v>
+      </c>
+      <c r="E108" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="F108" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="109" ht="42" customHeight="1">
+      <c r="A109" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B109" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:JQOojiI6XY0C</t>
+        </is>
+      </c>
+      <c r="C109" s="20" t="inlineStr">
+        <is>
+          <t>Temcoco: Temporally consistent multi-modal video fusion with visual-semantic collaboration</t>
+        </is>
+      </c>
+      <c r="D109" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="E109" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F109" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="110" ht="42" customHeight="1">
+      <c r="A110" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B110" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:Y5dfb0dijaUC</t>
+        </is>
+      </c>
+      <c r="C110" s="20" t="inlineStr">
+        <is>
+          <t>Text-if: Leveraging semantic text guidance for degradation-aware and interactive image fusion</t>
+        </is>
+      </c>
+      <c r="D110" s="16" t="n">
+        <v>376</v>
+      </c>
+      <c r="E110" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F110" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="111" ht="42" customHeight="1">
+      <c r="A111" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B111" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:evX43VCCuoAC</t>
+        </is>
+      </c>
+      <c r="C111" s="20" t="inlineStr">
+        <is>
+          <t>Videofusion: a spatio-temporal collaborative network for multi-modal video fusion</t>
+        </is>
+      </c>
+      <c r="D111" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="E111" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" s="17" t="n">
+        <v>46296.66398726479</v>
+      </c>
+    </row>
+    <row r="112" ht="42" customHeight="1">
+      <c r="A112" s="18" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B112" s="19" t="inlineStr">
+        <is>
+          <t>PyRqpAsAAAAJ:NJ774b8OgUMC</t>
+        </is>
+      </c>
+      <c r="C112" s="20" t="inlineStr">
+        <is>
+          <t>基于深度学习的图像融合方法综述</t>
+        </is>
+      </c>
+      <c r="D112" s="16" t="n">
+        <v>39</v>
+      </c>
+      <c r="E112" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F112" s="17" t="n">
+        <v>46296.66398726479</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F75"/>
+  <autoFilter ref="A1:F112"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>